<commit_message>
atualiza volumes loa com ppo - 21092026.2
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -7831,21 +7831,21 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E323" t="n">
-        <v>1703</v>
+        <v>3</v>
       </c>
     </row>
     <row r="324">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -7864,11 +7864,11 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E324" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="325">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -7887,11 +7887,11 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>4</v>
+        <v>68</v>
       </c>
     </row>
     <row r="326">
@@ -7900,21 +7900,21 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="327">
@@ -7923,21 +7923,21 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>11</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="328">
@@ -7951,16 +7951,16 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E328" t="n">
-        <v>82</v>
+        <v>3</v>
       </c>
     </row>
     <row r="329">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -7979,11 +7979,11 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E329" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="330">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -8002,11 +8002,11 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E330" t="n">
-        <v>4125</v>
+        <v>25</v>
       </c>
     </row>
     <row r="331">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -8025,11 +8025,11 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>21486</v>
+        <v>11</v>
       </c>
     </row>
     <row r="332">
@@ -8038,21 +8038,21 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>14673</v>
+        <v>82</v>
       </c>
     </row>
     <row r="333">
@@ -8071,11 +8071,11 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>155811</v>
+        <v>6</v>
       </c>
     </row>
     <row r="334">
@@ -8094,11 +8094,11 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>39906</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="335">
@@ -8112,15 +8112,107 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
+      <c r="D339" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E335" t="n">
+      <c r="E339" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 22092026.2
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -3719,16 +3719,16 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>7</v>
+        <v>315</v>
       </c>
     </row>
     <row r="145">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2351 - UEMG</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3747,11 +3747,11 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E145" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
     </row>
     <row r="146">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2351 - UEMG</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E146" t="n">
-        <v>399</v>
+        <v>663</v>
       </c>
     </row>
     <row r="147">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2351 - UEMG</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3793,11 +3793,11 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>1784</v>
+        <v>313</v>
       </c>
     </row>
     <row r="148">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2351 - UEMG</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3820,7 +3820,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>175</v>
+        <v>133</v>
       </c>
     </row>
     <row r="149">
@@ -3829,21 +3829,21 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2351 - UEMG</t>
+          <t>1501 - SEPLAG</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E149" t="n">
-        <v>505</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="150">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -3866,7 +3866,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="151">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -3889,7 +3889,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>663</v>
+        <v>29</v>
       </c>
     </row>
     <row r="152">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E152" t="n">
-        <v>313</v>
+        <v>43</v>
       </c>
     </row>
     <row r="153">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3931,11 +3931,11 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>133</v>
+        <v>99</v>
       </c>
     </row>
     <row r="154">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>1501 - SEPLAG</t>
+          <t>2241 - IGAM</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3958,7 +3958,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>1529</v>
+        <v>51</v>
       </c>
     </row>
     <row r="155">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -4004,7 +4004,7 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="157">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4023,11 +4023,11 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
     </row>
     <row r="158">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4046,11 +4046,11 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E158" t="n">
-        <v>99</v>
+        <v>258</v>
       </c>
     </row>
     <row r="159">
@@ -4059,21 +4059,21 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2241 - IGAM</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>NATUREZA ESPECIAL</t>
         </is>
       </c>
       <c r="E159" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -4092,11 +4092,11 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E160" t="n">
-        <v>1</v>
+        <v>243</v>
       </c>
     </row>
     <row r="161">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>1251 - PMMG</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>32</v>
+        <v>2855</v>
       </c>
     </row>
     <row r="162">
@@ -4138,11 +4138,11 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E162" t="n">
-        <v>3</v>
+        <v>1828</v>
       </c>
     </row>
     <row r="163">
@@ -4161,11 +4161,11 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>258</v>
+        <v>3483</v>
       </c>
     </row>
     <row r="164">
@@ -4184,11 +4184,11 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>NATUREZA ESPECIAL</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>1</v>
+        <v>34165</v>
       </c>
     </row>
     <row r="165">
@@ -4202,16 +4202,16 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E165" t="n">
-        <v>243</v>
+        <v>874</v>
       </c>
     </row>
     <row r="166">
@@ -4225,16 +4225,16 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>2855</v>
+        <v>38749</v>
       </c>
     </row>
     <row r="167">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E167" t="n">
-        <v>1828</v>
+        <v>3</v>
       </c>
     </row>
     <row r="168">
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4276,11 +4276,11 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E168" t="n">
-        <v>3483</v>
+        <v>22</v>
       </c>
     </row>
     <row r="169">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4299,11 +4299,11 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E169" t="n">
-        <v>34165</v>
+        <v>83</v>
       </c>
     </row>
     <row r="170">
@@ -4312,21 +4312,21 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>2331 - IPEMMG</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>874</v>
+        <v>13</v>
       </c>
     </row>
     <row r="171">
@@ -4335,21 +4335,21 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>1251 - PMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>38749</v>
+        <v>22</v>
       </c>
     </row>
     <row r="172">
@@ -4363,16 +4363,16 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>3</v>
+        <v>151</v>
       </c>
     </row>
     <row r="173">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4391,11 +4391,11 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E173" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4414,11 +4414,11 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E174" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
     </row>
     <row r="175">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4437,11 +4437,11 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="176">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E176" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
     </row>
     <row r="177">
@@ -4473,21 +4473,21 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2331 - IPEMMG</t>
+          <t>2201 - IEPHA</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E177" t="n">
-        <v>151</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4506,11 +4506,11 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E178" t="n">
-        <v>1</v>
+        <v>135</v>
       </c>
     </row>
     <row r="179">
@@ -4524,16 +4524,16 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>22</v>
+        <v>65</v>
       </c>
     </row>
     <row r="180">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4552,11 +4552,11 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="181">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4575,11 +4575,11 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>45</v>
+        <v>22</v>
       </c>
     </row>
     <row r="182">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4598,11 +4598,11 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OFICIAL</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>1</v>
+        <v>794</v>
       </c>
     </row>
     <row r="183">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4621,11 +4621,11 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>PRAÇA</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>135</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="184">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2201 - IEPHA</t>
+          <t>1401 - CBMMG</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4644,11 +4644,11 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>INATIVO MILITAR</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>65</v>
+        <v>3190</v>
       </c>
     </row>
     <row r="185">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4694,7 +4694,7 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>22</v>
+        <v>41</v>
       </c>
     </row>
     <row r="187">
@@ -4703,21 +4703,21 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>OFICIAL</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>794</v>
+        <v>10</v>
       </c>
     </row>
     <row r="188">
@@ -4726,21 +4726,21 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>1521 - CGE</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>PRAÇA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>5154</v>
+        <v>19</v>
       </c>
     </row>
     <row r="189">
@@ -4749,21 +4749,21 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>1401 - CBMMG</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>INATIVO MILITAR</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>3190</v>
+        <v>5</v>
       </c>
     </row>
     <row r="190">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -4782,11 +4782,11 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>2</v>
+        <v>769</v>
       </c>
     </row>
     <row r="191">
@@ -4795,7 +4795,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>41</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="192">
@@ -4818,21 +4818,21 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>10</v>
+        <v>533</v>
       </c>
     </row>
     <row r="193">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>1521 - CGE</t>
+          <t>1191 - SEF</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4855,7 +4855,7 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>19</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="194">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4901,7 +4901,7 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>769</v>
+        <v>117</v>
       </c>
     </row>
     <row r="196">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4920,11 +4920,11 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>1440</v>
+        <v>17</v>
       </c>
     </row>
     <row r="197">
@@ -4933,7 +4933,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4943,11 +4943,11 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>533</v>
+        <v>17</v>
       </c>
     </row>
     <row r="198">
@@ -4956,21 +4956,21 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>1191 - SEF</t>
+          <t>1231 - SEAPA</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>4251</v>
+        <v>31</v>
       </c>
     </row>
     <row r="199">
@@ -4984,16 +4984,16 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>5</v>
+        <v>317</v>
       </c>
     </row>
     <row r="200">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5012,11 +5012,11 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>117</v>
+        <v>43</v>
       </c>
     </row>
     <row r="201">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -5035,11 +5035,11 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>17</v>
+        <v>295</v>
       </c>
     </row>
     <row r="202">
@@ -5048,7 +5048,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>17</v>
+        <v>120</v>
       </c>
     </row>
     <row r="203">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>3051 - EPAMIG</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -5081,11 +5081,11 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>31</v>
+        <v>175</v>
       </c>
     </row>
     <row r="204">
@@ -5094,21 +5094,21 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>1231 - SEAPA</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>317</v>
+        <v>7</v>
       </c>
     </row>
     <row r="205">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -5127,11 +5127,11 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="206">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>295</v>
+        <v>121</v>
       </c>
     </row>
     <row r="207">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5177,7 +5177,7 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>120</v>
+        <v>85</v>
       </c>
     </row>
     <row r="208">
@@ -5186,21 +5186,21 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>3051 - EPAMIG</t>
+          <t>1301 - SEINFRA</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>175</v>
+        <v>71</v>
       </c>
     </row>
     <row r="209">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="210">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5246,7 +5246,7 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
     </row>
     <row r="211">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5265,11 +5265,11 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>121</v>
+        <v>94</v>
       </c>
     </row>
     <row r="212">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5288,11 +5288,11 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E212" t="n">
-        <v>85</v>
+        <v>25</v>
       </c>
     </row>
     <row r="213">
@@ -5301,21 +5301,21 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>1301 - SEINFRA</t>
+          <t>2251 - JUCEMG</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>71</v>
+        <v>12</v>
       </c>
     </row>
     <row r="214">
@@ -5334,11 +5334,11 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
     </row>
     <row r="215">
@@ -5352,16 +5352,16 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>27</v>
+        <v>124</v>
       </c>
     </row>
     <row r="216">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>2281 - UTRAMIG</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5380,11 +5380,11 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>94</v>
+        <v>10</v>
       </c>
     </row>
     <row r="217">
@@ -5393,7 +5393,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>2281 - UTRAMIG</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5403,11 +5403,11 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="218">
@@ -5416,7 +5416,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5426,11 +5426,11 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E218" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="219">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5449,11 +5449,11 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="220">
@@ -5462,21 +5462,21 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2251 - JUCEMG</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>124</v>
+        <v>898</v>
       </c>
     </row>
     <row r="221">
@@ -5485,7 +5485,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2281 - UTRAMIG</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="222">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2281 - UTRAMIG</t>
+          <t>2371 - IMA</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5518,11 +5518,11 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>7</v>
+        <v>343</v>
       </c>
     </row>
     <row r="223">
@@ -5536,16 +5536,16 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>4</v>
+        <v>595</v>
       </c>
     </row>
     <row r="224">
@@ -5559,16 +5559,16 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E224" t="n">
-        <v>38</v>
+        <v>48</v>
       </c>
     </row>
     <row r="225">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -5587,11 +5587,11 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E225" t="n">
-        <v>898</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -5610,11 +5610,11 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E226" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="227">
@@ -5623,7 +5623,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E227" t="n">
-        <v>343</v>
+        <v>224</v>
       </c>
     </row>
     <row r="228">
@@ -5646,21 +5646,21 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E228" t="n">
-        <v>595</v>
+        <v>282</v>
       </c>
     </row>
     <row r="229">
@@ -5669,21 +5669,21 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2371 - IMA</t>
+          <t>2261 - FUNED</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E229" t="n">
-        <v>48</v>
+        <v>183</v>
       </c>
     </row>
     <row r="230">
@@ -5697,16 +5697,16 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E230" t="n">
-        <v>1</v>
+        <v>276</v>
       </c>
     </row>
     <row r="231">
@@ -5715,7 +5715,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -5725,11 +5725,11 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E231" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="232">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5748,11 +5748,11 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>224</v>
+        <v>946</v>
       </c>
     </row>
     <row r="233">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5775,7 +5775,7 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>282</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="234">
@@ -5784,7 +5784,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5798,7 +5798,7 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>183</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="235">
@@ -5807,21 +5807,21 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2261 - FUNED</t>
+          <t>1091 - PGJ</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>276</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="236">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -5840,11 +5840,11 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">
@@ -5858,16 +5858,16 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>946</v>
+        <v>829</v>
       </c>
     </row>
     <row r="238">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5886,11 +5886,11 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>1350</v>
+        <v>33</v>
       </c>
     </row>
     <row r="239">
@@ -5899,7 +5899,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5909,11 +5909,11 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>1351</v>
+        <v>75</v>
       </c>
     </row>
     <row r="240">
@@ -5922,7 +5922,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5932,11 +5932,11 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>1138</v>
+        <v>364</v>
       </c>
     </row>
     <row r="241">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5959,7 +5959,7 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>1</v>
+        <v>534</v>
       </c>
     </row>
     <row r="242">
@@ -5968,21 +5968,21 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>1091 - PGJ</t>
+          <t>1011 - ALMG</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E242" t="n">
-        <v>829</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="243">
@@ -6001,11 +6001,11 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E243" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="244">
@@ -6024,11 +6024,11 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E244" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="245">
@@ -6042,16 +6042,16 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E245" t="n">
-        <v>364</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="246">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -6070,11 +6070,11 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E246" t="n">
-        <v>534</v>
+        <v>2</v>
       </c>
     </row>
     <row r="247">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6093,11 +6093,11 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E247" t="n">
-        <v>2500</v>
+        <v>91</v>
       </c>
     </row>
     <row r="248">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>1711 - SECOM</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6116,11 +6116,11 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E248" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
     </row>
     <row r="249">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>2431 - AGÊNCIA RMBH</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -6139,11 +6139,11 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E249" t="n">
-        <v>77</v>
+        <v>1</v>
       </c>
     </row>
     <row r="250">
@@ -6152,21 +6152,21 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>1011 - ALMG</t>
+          <t>2431 - AGÊNCIA RMBH</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>1251</v>
+        <v>9</v>
       </c>
     </row>
     <row r="251">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>2431 - AGÊNCIA RMBH</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -6185,11 +6185,11 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
     </row>
     <row r="252">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>91</v>
+        <v>8</v>
       </c>
     </row>
     <row r="253">
@@ -6221,7 +6221,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>1711 - SECOM</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -6231,11 +6231,11 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
     </row>
     <row r="254">
@@ -6244,7 +6244,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2431 - AGÊNCIA RMBH</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
@@ -6254,11 +6254,11 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>1</v>
+        <v>131</v>
       </c>
     </row>
     <row r="255">
@@ -6267,21 +6267,21 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2431 - AGÊNCIA RMBH</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="256">
@@ -6290,21 +6290,21 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2431 - AGÊNCIA RMBH</t>
+          <t>1221 - SEDE</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>23</v>
+        <v>398</v>
       </c>
     </row>
     <row r="257">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="E257" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>53</v>
+        <v>78</v>
       </c>
     </row>
     <row r="259">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6369,11 +6369,11 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>131</v>
+        <v>54</v>
       </c>
     </row>
     <row r="260">
@@ -6382,21 +6382,21 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>2</v>
+        <v>286</v>
       </c>
     </row>
     <row r="261">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>1221 - SEDE</t>
+          <t>2091 - FEAM</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="E261" t="n">
-        <v>398</v>
+        <v>95</v>
       </c>
     </row>
     <row r="262">
@@ -6428,7 +6428,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E262" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="263">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -6465,7 +6465,7 @@
         </is>
       </c>
       <c r="E263" t="n">
-        <v>78</v>
+        <v>613</v>
       </c>
     </row>
     <row r="264">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -6488,7 +6488,7 @@
         </is>
       </c>
       <c r="E264" t="n">
-        <v>54</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="265">
@@ -6497,7 +6497,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
@@ -6511,7 +6511,7 @@
         </is>
       </c>
       <c r="E265" t="n">
-        <v>286</v>
+        <v>4354</v>
       </c>
     </row>
     <row r="266">
@@ -6520,21 +6520,21 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2091 - FEAM</t>
+          <t>2271 - FHEMIG</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>95</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="267">
@@ -6553,11 +6553,11 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>2</v>
+        <v>844</v>
       </c>
     </row>
     <row r="268">
@@ -6571,16 +6571,16 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>613</v>
+        <v>4085</v>
       </c>
     </row>
     <row r="269">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -6599,11 +6599,11 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>5712</v>
+        <v>2</v>
       </c>
     </row>
     <row r="270">
@@ -6612,7 +6612,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -6622,11 +6622,11 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>4354</v>
+        <v>61</v>
       </c>
     </row>
     <row r="271">
@@ -6635,7 +6635,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -6645,11 +6645,11 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>1146</v>
+        <v>36</v>
       </c>
     </row>
     <row r="272">
@@ -6658,7 +6658,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -6668,11 +6668,11 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>844</v>
+        <v>147</v>
       </c>
     </row>
     <row r="273">
@@ -6681,21 +6681,21 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2271 - FHEMIG</t>
+          <t>2061 - FJP</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>4085</v>
+        <v>3</v>
       </c>
     </row>
     <row r="274">
@@ -6714,11 +6714,11 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="275">
@@ -6732,16 +6732,16 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>61</v>
+        <v>283</v>
       </c>
     </row>
     <row r="276">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6760,11 +6760,11 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
     </row>
     <row r="277">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>147</v>
+        <v>4</v>
       </c>
     </row>
     <row r="278">
@@ -6796,7 +6796,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -6806,11 +6806,11 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>3</v>
+        <v>513</v>
       </c>
     </row>
     <row r="279">
@@ -6819,7 +6819,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>3041 - EMATER</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -6829,11 +6829,11 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>1</v>
+        <v>863</v>
       </c>
     </row>
     <row r="280">
@@ -6842,21 +6842,21 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2061 - FJP</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>283</v>
+        <v>149</v>
       </c>
     </row>
     <row r="281">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2481 - DETRANMG</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -6875,11 +6875,11 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>3</v>
+        <v>38</v>
       </c>
     </row>
     <row r="282">
@@ -6888,7 +6888,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -6898,11 +6898,11 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
@@ -6911,7 +6911,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6921,11 +6921,11 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>513</v>
+        <v>217</v>
       </c>
     </row>
     <row r="284">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>3041 - EMATER</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
@@ -6944,11 +6944,11 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>863</v>
+        <v>227</v>
       </c>
     </row>
     <row r="285">
@@ -6957,7 +6957,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -6971,7 +6971,7 @@
         </is>
       </c>
       <c r="E285" t="n">
-        <v>149</v>
+        <v>296</v>
       </c>
     </row>
     <row r="286">
@@ -6980,21 +6980,21 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2481 - DETRANMG</t>
+          <t>2101 - IEF</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Mão De Obra Temporária</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TERCEIRIZADO</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
     </row>
     <row r="287">
@@ -7008,16 +7008,16 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>1</v>
+        <v>411</v>
       </c>
     </row>
     <row r="288">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2101 - IEF</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7036,11 +7036,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>217</v>
+        <v>5</v>
       </c>
     </row>
     <row r="289">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2101 - IEF</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7059,11 +7059,11 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>227</v>
+        <v>3781</v>
       </c>
     </row>
     <row r="290">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2101 - IEF</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -7082,11 +7082,11 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>296</v>
+        <v>107</v>
       </c>
     </row>
     <row r="291">
@@ -7095,21 +7095,21 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2101 - IEF</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Mão De Obra Temporária</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>TERCEIRIZADO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>10</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="292">
@@ -7118,21 +7118,21 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2101 - IEF</t>
+          <t>4031 - FEPJ</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>411</v>
+        <v>8398</v>
       </c>
     </row>
     <row r="293">
@@ -7151,11 +7151,11 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>5</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="294">
@@ -7169,16 +7169,16 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>3781</v>
+        <v>6858</v>
       </c>
     </row>
     <row r="295">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7197,11 +7197,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>107</v>
+        <v>4</v>
       </c>
     </row>
     <row r="296">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>1258</v>
+        <v>158</v>
       </c>
     </row>
     <row r="297">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>8398</v>
+        <v>56</v>
       </c>
     </row>
     <row r="298">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7266,11 +7266,11 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>1085</v>
+        <v>38</v>
       </c>
     </row>
     <row r="299">
@@ -7279,21 +7279,21 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>6858</v>
+        <v>1</v>
       </c>
     </row>
     <row r="300">
@@ -7307,16 +7307,16 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>4</v>
+        <v>273</v>
       </c>
     </row>
     <row r="301">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>158</v>
+        <v>7</v>
       </c>
     </row>
     <row r="302">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
     </row>
     <row r="303">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
     </row>
     <row r="304">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
     </row>
     <row r="305">
@@ -7417,21 +7417,21 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>273</v>
+        <v>282</v>
       </c>
     </row>
     <row r="306">
@@ -7450,11 +7450,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>7</v>
+        <v>205</v>
       </c>
     </row>
     <row r="307">
@@ -7468,16 +7468,16 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>13</v>
+        <v>53</v>
       </c>
     </row>
     <row r="308">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7496,11 +7496,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="309">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7519,11 +7519,11 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>48</v>
+        <v>18</v>
       </c>
     </row>
     <row r="310">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7542,11 +7542,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>282</v>
+        <v>17</v>
       </c>
     </row>
     <row r="311">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7569,7 +7569,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>205</v>
+        <v>17</v>
       </c>
     </row>
     <row r="312">
@@ -7578,21 +7578,21 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
     </row>
     <row r="313">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7611,11 +7611,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="314">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7634,11 +7634,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>18</v>
+        <v>56</v>
       </c>
     </row>
     <row r="315">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -7657,11 +7657,11 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="316">
@@ -7670,21 +7670,21 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="317">
@@ -7923,21 +7923,21 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>1703</v>
+        <v>1</v>
       </c>
     </row>
     <row r="328">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -7956,11 +7956,11 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E328" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="329">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -7979,11 +7979,11 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E329" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="330">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -8002,11 +8002,11 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E330" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="331">
@@ -8015,21 +8015,21 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="332">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -8052,7 +8052,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>82</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="333">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -8075,7 +8075,7 @@
         </is>
       </c>
       <c r="E333" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="334">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8098,7 +8098,7 @@
         </is>
       </c>
       <c r="E334" t="n">
-        <v>4125</v>
+        <v>4</v>
       </c>
     </row>
     <row r="335">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -8121,7 +8121,7 @@
         </is>
       </c>
       <c r="E335" t="n">
-        <v>21486</v>
+        <v>25</v>
       </c>
     </row>
     <row r="336">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -8140,11 +8140,11 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>14673</v>
+        <v>11</v>
       </c>
     </row>
     <row r="337">
@@ -8153,21 +8153,21 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E337" t="n">
-        <v>155811</v>
+        <v>82</v>
       </c>
     </row>
     <row r="338">
@@ -8186,11 +8186,11 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E338" t="n">
-        <v>39906</v>
+        <v>6</v>
       </c>
     </row>
     <row r="339">
@@ -8204,15 +8204,130 @@
       </c>
       <c r="C339" t="inlineStr">
         <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
+      <c r="D344" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E339" t="n">
+      <c r="E344" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 23092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -7026,7 +7026,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7040,7 +7040,7 @@
         </is>
       </c>
       <c r="E288" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="289">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="E289" t="n">
-        <v>3781</v>
+        <v>158</v>
       </c>
     </row>
     <row r="290">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -7086,7 +7086,7 @@
         </is>
       </c>
       <c r="E290" t="n">
-        <v>107</v>
+        <v>56</v>
       </c>
     </row>
     <row r="291">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -7109,7 +7109,7 @@
         </is>
       </c>
       <c r="E291" t="n">
-        <v>1258</v>
+        <v>38</v>
       </c>
     </row>
     <row r="292">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -7128,11 +7128,11 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>8398</v>
+        <v>1</v>
       </c>
     </row>
     <row r="293">
@@ -7141,21 +7141,21 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>MEMBROS DE PODER</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>1085</v>
+        <v>273</v>
       </c>
     </row>
     <row r="294">
@@ -7164,21 +7164,21 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>4031 - FEPJ</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>6858</v>
+        <v>7</v>
       </c>
     </row>
     <row r="295">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7197,11 +7197,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="296">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>158</v>
+        <v>22</v>
       </c>
     </row>
     <row r="297">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
     </row>
     <row r="298">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7266,11 +7266,11 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>38</v>
+        <v>282</v>
       </c>
     </row>
     <row r="299">
@@ -7279,7 +7279,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>1</v>
+        <v>205</v>
       </c>
     </row>
     <row r="300">
@@ -7302,7 +7302,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7316,7 +7316,7 @@
         </is>
       </c>
       <c r="E300" t="n">
-        <v>273</v>
+        <v>53</v>
       </c>
     </row>
     <row r="301">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7339,7 +7339,7 @@
         </is>
       </c>
       <c r="E301" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="302">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="E302" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="303">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="304">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7404,11 +7404,11 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
     </row>
     <row r="305">
@@ -7417,7 +7417,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7427,11 +7427,11 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>282</v>
+        <v>1</v>
       </c>
     </row>
     <row r="306">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7450,11 +7450,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>205</v>
+        <v>13</v>
       </c>
     </row>
     <row r="307">
@@ -7463,21 +7463,21 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="308">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7496,11 +7496,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="309">
@@ -7509,21 +7509,21 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="310">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7542,11 +7542,11 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="311">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7565,11 +7565,11 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="312">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -7588,11 +7588,11 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="313">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7611,11 +7611,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="314">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7634,11 +7634,11 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="315">
@@ -7647,21 +7647,21 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="316">
@@ -7670,21 +7670,21 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="317">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E317" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
     </row>
     <row r="318">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7726,11 +7726,11 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>24</v>
+        <v>68</v>
       </c>
     </row>
     <row r="319">
@@ -7739,21 +7739,21 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E319" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="320">
@@ -7762,7 +7762,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -7772,11 +7772,11 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="321">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="322">
@@ -7808,21 +7808,21 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
     </row>
     <row r="323">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -7841,11 +7841,11 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E323" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="324">
@@ -7854,21 +7854,21 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E324" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
     </row>
     <row r="325">
@@ -7877,21 +7877,21 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>1941 - EGE-SEPLAG</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>68</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="326">
@@ -7900,17 +7900,17 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E326" t="n">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="328">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -7956,11 +7956,11 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E328" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="329">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -7979,11 +7979,11 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E329" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="330">
@@ -7992,21 +7992,21 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E330" t="n">
-        <v>13</v>
+        <v>82</v>
       </c>
     </row>
     <row r="331">
@@ -8015,21 +8015,21 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="332">
@@ -8038,21 +8038,21 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>1703</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="333">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -8071,11 +8071,11 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>3</v>
+        <v>21486</v>
       </c>
     </row>
     <row r="334">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8094,11 +8094,11 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>4</v>
+        <v>14673</v>
       </c>
     </row>
     <row r="335">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -8117,11 +8117,11 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>25</v>
+        <v>155811</v>
       </c>
     </row>
     <row r="336">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -8144,7 +8144,7 @@
         </is>
       </c>
       <c r="E336" t="n">
-        <v>11</v>
+        <v>39906</v>
       </c>
     </row>
     <row r="337">
@@ -8153,7 +8153,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -8167,167 +8167,6 @@
         </is>
       </c>
       <c r="E337" t="n">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>DIREÇÃO SUPERIOR</t>
-        </is>
-      </c>
-      <c r="E338" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
-        </is>
-      </c>
-      <c r="E339" t="n">
-        <v>4125</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>TÉCNICA</t>
-        </is>
-      </c>
-      <c r="E340" t="n">
-        <v>21486</v>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D341" t="inlineStr">
-        <is>
-          <t>ESPECIALIZADA</t>
-        </is>
-      </c>
-      <c r="E341" t="n">
-        <v>14673</v>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>DOCENTE</t>
-        </is>
-      </c>
-      <c r="E342" t="n">
-        <v>155811</v>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>ADMINISTRATIVA</t>
-        </is>
-      </c>
-      <c r="E343" t="n">
-        <v>39906</v>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t>Inativo</t>
-        </is>
-      </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>INATIVO CIVIL</t>
-        </is>
-      </c>
-      <c r="E344" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 23092026.2
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -7877,21 +7877,21 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>1941 - EGE-SEPLAG</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>1703</v>
+        <v>3</v>
       </c>
     </row>
     <row r="326">
@@ -7910,11 +7910,11 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="327">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="328">
@@ -7956,11 +7956,11 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E328" t="n">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="329">
@@ -7974,16 +7974,16 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E329" t="n">
-        <v>11</v>
+        <v>82</v>
       </c>
     </row>
     <row r="330">
@@ -7992,21 +7992,21 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>1261 - SEE</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E330" t="n">
-        <v>82</v>
+        <v>6</v>
       </c>
     </row>
     <row r="331">
@@ -8025,11 +8025,11 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E331" t="n">
-        <v>6</v>
+        <v>4125</v>
       </c>
     </row>
     <row r="332">
@@ -8048,11 +8048,11 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E332" t="n">
-        <v>4125</v>
+        <v>21486</v>
       </c>
     </row>
     <row r="333">
@@ -8071,11 +8071,11 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>21486</v>
+        <v>14673</v>
       </c>
     </row>
     <row r="334">
@@ -8094,11 +8094,11 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>14673</v>
+        <v>155811</v>
       </c>
     </row>
     <row r="335">
@@ -8117,11 +8117,11 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>155811</v>
+        <v>39906</v>
       </c>
     </row>
     <row r="336">
@@ -8135,38 +8135,15 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E336" t="n">
-        <v>39906</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>1261 - SEE</t>
-        </is>
-      </c>
-      <c r="C337" t="inlineStr">
-        <is>
-          <t>Inativo</t>
-        </is>
-      </c>
-      <c r="D337" t="inlineStr">
-        <is>
-          <t>INATIVO CIVIL</t>
-        </is>
-      </c>
-      <c r="E337" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualiza volumes loa com ppo - 24092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
+++ b/bancos/SISOR/BASE_CATEGORIA_PESSOAL.xlsx
@@ -7026,7 +7026,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>1021 - TCEMG</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7036,11 +7036,11 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>4</v>
+        <v>225</v>
       </c>
     </row>
     <row r="289">
@@ -7049,7 +7049,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>1021 - TCEMG</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -7059,11 +7059,11 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>158</v>
+        <v>825</v>
       </c>
     </row>
     <row r="290">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>1021 - TCEMG</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -7082,11 +7082,11 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>56</v>
+        <v>245</v>
       </c>
     </row>
     <row r="291">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>1021 - TCEMG</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -7105,11 +7105,11 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>MEMBROS DE PODER</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>38</v>
+        <v>15</v>
       </c>
     </row>
     <row r="292">
@@ -7118,21 +7118,21 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>1271 - SECULT</t>
+          <t>1021 - TCEMG</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>OUTRAS</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>1</v>
+        <v>845</v>
       </c>
     </row>
     <row r="293">
@@ -7146,16 +7146,16 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>273</v>
+        <v>4</v>
       </c>
     </row>
     <row r="294">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -7174,11 +7174,11 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>7</v>
+        <v>158</v>
       </c>
     </row>
     <row r="295">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -7197,11 +7197,11 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
     </row>
     <row r="296">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7220,11 +7220,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
     </row>
     <row r="297">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7243,11 +7243,11 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>OUTRAS</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>48</v>
+        <v>1</v>
       </c>
     </row>
     <row r="298">
@@ -7256,21 +7256,21 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2151 - FHA</t>
+          <t>1271 - SECULT</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="299">
@@ -7289,11 +7289,11 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>205</v>
+        <v>7</v>
       </c>
     </row>
     <row r="300">
@@ -7307,16 +7307,16 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
     </row>
     <row r="301">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7335,11 +7335,11 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="302">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
     </row>
     <row r="303">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7381,11 +7381,11 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>17</v>
+        <v>282</v>
       </c>
     </row>
     <row r="304">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2471 - ARTEMIG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7408,7 +7408,7 @@
         </is>
       </c>
       <c r="E304" t="n">
-        <v>17</v>
+        <v>205</v>
       </c>
     </row>
     <row r="305">
@@ -7417,21 +7417,21 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2151 - FHA</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>1</v>
+        <v>53</v>
       </c>
     </row>
     <row r="306">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7450,11 +7450,11 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="307">
@@ -7463,7 +7463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7473,11 +7473,11 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>56</v>
+        <v>18</v>
       </c>
     </row>
     <row r="308">
@@ -7486,7 +7486,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7496,11 +7496,11 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="309">
@@ -7509,21 +7509,21 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>1541 - ESP MG</t>
+          <t>2471 - ARTEMIG</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="310">
@@ -7532,7 +7532,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7555,7 +7555,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7569,7 +7569,7 @@
         </is>
       </c>
       <c r="E311" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="312">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -7588,11 +7588,11 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>16</v>
+        <v>56</v>
       </c>
     </row>
     <row r="313">
@@ -7601,7 +7601,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -7611,11 +7611,11 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="314">
@@ -7624,21 +7624,21 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2421 - IDENE</t>
+          <t>1541 - ESP MG</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
     </row>
     <row r="315">
@@ -7652,16 +7652,16 @@
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
     </row>
     <row r="316">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -7680,11 +7680,11 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="317">
@@ -7693,7 +7693,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -7703,11 +7703,11 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>TÉCNICA</t>
         </is>
       </c>
       <c r="E317" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="318">
@@ -7716,7 +7716,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7726,11 +7726,11 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>ESPECIALIZADA</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>68</v>
+        <v>32</v>
       </c>
     </row>
     <row r="319">
@@ -7739,21 +7739,21 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>1101 - OGE</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Inativo</t>
+          <t>Ativo</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>INATIVO CIVIL</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E319" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="320">
@@ -7762,21 +7762,21 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>2421 - IDENE</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>DIREÇÃO SUPERIOR</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="321">
@@ -7785,7 +7785,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -7795,11 +7795,11 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>DIREÇÃO E ASSESSORAMENTO</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="322">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -7818,11 +7818,11 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="323">
@@ -7831,7 +7831,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -7845,7 +7845,7 @@
         </is>
       </c>
       <c r="E323" t="n">
-        <v>13</v>
+        <v>68</v>
       </c>
     </row>
     <row r="324">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2171 - FAOP</t>
+          <t>1101 - OGE</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -7868,7 +7868,7 @@
         </is>
       </c>
       <c r="E324" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="325">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -7891,7 +7891,7 @@
         </is>
       </c>
       <c r="E325" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="326">
@@ -7900,7 +7900,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="E326" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="327">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -7933,11 +7933,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>TÉCNICA</t>
+          <t>DOCENTE</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="328">
@@ -7946,7 +7946,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="E328" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="329">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2161 - FUCAM</t>
+          <t>2171 - FAOP</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -7983,7 +7983,7 @@
         </is>
       </c>
       <c r="E329" t="n">
-        <v>82</v>
+        <v>4</v>
       </c>
     </row>
     <row r="330">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -8006,7 +8006,7 @@
         </is>
       </c>
       <c r="E330" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="331">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -8029,7 +8029,7 @@
         </is>
       </c>
       <c r="E331" t="n">
-        <v>4125</v>
+        <v>4</v>
       </c>
     </row>
     <row r="332">
@@ -8038,7 +8038,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -8052,7 +8052,7 @@
         </is>
       </c>
       <c r="E332" t="n">
-        <v>21486</v>
+        <v>25</v>
       </c>
     </row>
     <row r="333">
@@ -8061,7 +8061,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -8071,11 +8071,11 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>ESPECIALIZADA</t>
+          <t>ADMINISTRATIVA</t>
         </is>
       </c>
       <c r="E333" t="n">
-        <v>14673</v>
+        <v>11</v>
       </c>
     </row>
     <row r="334">
@@ -8084,21 +8084,21 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>1261 - SEE</t>
+          <t>2161 - FUCAM</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Inativo</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>DOCENTE</t>
+          <t>INATIVO CIVIL</t>
         </is>
       </c>
       <c r="E334" t="n">
-        <v>155811</v>
+        <v>82</v>
       </c>
     </row>
     <row r="335">
@@ -8117,11 +8117,11 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>ADMINISTRATIVA</t>
+          <t>DIREÇÃO SUPERIOR</t>
         </is>
       </c>
       <c r="E335" t="n">
-        <v>39906</v>
+        <v>6</v>
       </c>
     </row>
     <row r="336">
@@ -8135,15 +8135,130 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>DIREÇÃO E ASSESSORAMENTO</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>TÉCNICA</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>21486</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>ESPECIALIZADA</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>14673</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>DOCENTE</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>155811</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>39906</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>1261 - SEE</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
           <t>Inativo</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr">
+      <c r="D341" t="inlineStr">
         <is>
           <t>INATIVO CIVIL</t>
         </is>
       </c>
-      <c r="E336" t="n">
+      <c r="E341" t="n">
         <v>175450</v>
       </c>
     </row>

</xml_diff>